<commit_message>
Update settings, rates file; remove source PDF
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/260618_Seasonal rental Ratesxlsx.xlsx
+++ b/260618_Seasonal rental Ratesxlsx.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fd69bf0aab045e1c/Desktop/Claude Code/Nothing Quite Like It/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{65DAFD3D-EB96-4889-B122-CC1A0914954F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{150AA5FA-7F54-4BBC-9B7A-7052F184AB3A}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{65DAFD3D-EB96-4889-B122-CC1A0914954F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{023EB238-4673-43A0-82C9-6C97126706F8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{DF39FCA8-091E-470B-959D-C570A70A3390}"/>
   </bookViews>
@@ -39,15 +39,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t xml:space="preserve">  B.  WEEKLY GROSS RENT SCHEDULE  (sorted highest → lowest; model picks top N weeks for each scenario)</t>
   </si>
   <si>
     <t>Week / Season Category</t>
-  </si>
-  <si>
-    <t>Weekly Gross Rent (US$)</t>
   </si>
   <si>
     <t>Daily Gross Rent (US$)</t>
@@ -183,7 +180,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -216,13 +213,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -237,7 +227,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -254,12 +244,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE2E2E2"/>
         <bgColor rgb="FFF0F0F0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFDE7"/>
-        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -281,11 +265,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -298,11 +279,11 @@
     <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -638,503 +619,358 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B9E829C-EBAE-4761-A815-D354D0C5971D}">
-  <dimension ref="C5:E47"/>
+  <dimension ref="C5:D47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="44.6640625" customWidth="1"/>
-    <col min="4" max="5" width="13.6640625" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C5" s="1" t="s">
+    <row r="5" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C5" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="3:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="C6" s="2" t="s">
+      <c r="D5" s="6"/>
+    </row>
+    <row r="6" spans="3:4" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="C6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="3" t="s">
+    </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C7" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4">
+        <v>9429</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C8" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="5">
-        <v>66003</v>
-      </c>
-      <c r="E7" s="6">
-        <f t="shared" ref="E7:E47" si="0">D7/7</f>
-        <v>9429</v>
-      </c>
-    </row>
-    <row r="8" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="5">
-        <v>63000</v>
-      </c>
-      <c r="E8" s="6">
-        <f t="shared" si="0"/>
+      <c r="D9" s="4">
         <v>9000</v>
       </c>
     </row>
-    <row r="9" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C9" s="4" t="s">
+    <row r="10" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="5">
-        <v>63000</v>
-      </c>
-      <c r="E9" s="6">
-        <f t="shared" si="0"/>
+      <c r="D10" s="4">
         <v>9000</v>
       </c>
     </row>
-    <row r="10" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C10" s="4" t="s">
+    <row r="11" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C11" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="5">
-        <v>63000</v>
-      </c>
-      <c r="E10" s="6">
-        <f t="shared" si="0"/>
+      <c r="D11" s="4">
         <v>9000</v>
       </c>
     </row>
-    <row r="11" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C11" s="4" t="s">
+    <row r="12" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="5">
-        <v>63000</v>
-      </c>
-      <c r="E11" s="6">
-        <f t="shared" si="0"/>
+      <c r="D12" s="4">
         <v>9000</v>
       </c>
     </row>
-    <row r="12" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C12" s="4" t="s">
+    <row r="13" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="5">
-        <v>63000</v>
-      </c>
-      <c r="E12" s="6">
-        <f t="shared" si="0"/>
+      <c r="D13" s="4">
         <v>9000</v>
       </c>
     </row>
-    <row r="13" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C13" s="4" t="s">
+    <row r="14" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C14" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="5">
-        <v>63000</v>
-      </c>
-      <c r="E13" s="6">
-        <f t="shared" si="0"/>
+      <c r="D14" s="4">
         <v>9000</v>
       </c>
     </row>
-    <row r="14" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C14" s="4" t="s">
+    <row r="15" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C15" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="5">
-        <v>63000</v>
-      </c>
-      <c r="E14" s="6">
-        <f t="shared" si="0"/>
+      <c r="D15" s="4">
         <v>9000</v>
       </c>
     </row>
-    <row r="15" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C15" s="4" t="s">
+    <row r="16" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C16" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="5">
-        <v>63000</v>
-      </c>
-      <c r="E15" s="6">
-        <f t="shared" si="0"/>
+      <c r="D16" s="4">
         <v>9000</v>
       </c>
     </row>
-    <row r="16" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C16" s="4" t="s">
+    <row r="17" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C17" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="5">
-        <v>63000</v>
-      </c>
-      <c r="E16" s="6">
-        <f t="shared" si="0"/>
+      <c r="D17" s="4">
         <v>9000</v>
       </c>
     </row>
-    <row r="17" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C17" s="4" t="s">
+    <row r="18" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C18" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="5">
-        <v>63000</v>
-      </c>
-      <c r="E17" s="6">
-        <f t="shared" si="0"/>
-        <v>9000</v>
-      </c>
-    </row>
-    <row r="18" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C18" s="4" t="s">
+      <c r="D18" s="4">
+        <v>8999.8571428571431</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C19" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D18" s="5">
-        <v>62999</v>
-      </c>
-      <c r="E18" s="6">
-        <f t="shared" si="0"/>
-        <v>8999.8571428571431</v>
-      </c>
-    </row>
-    <row r="19" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C19" s="4" t="s">
+      <c r="D19" s="4">
+        <v>8571.4285714285706</v>
+      </c>
+    </row>
+    <row r="20" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C20" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D19" s="5">
-        <v>60000</v>
-      </c>
-      <c r="E19" s="6">
-        <f t="shared" si="0"/>
-        <v>8571.4285714285706</v>
-      </c>
-    </row>
-    <row r="20" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C20" s="4" t="s">
+      <c r="D20" s="4">
+        <v>8500</v>
+      </c>
+    </row>
+    <row r="21" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C21" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D20" s="5">
-        <v>59500</v>
-      </c>
-      <c r="E20" s="6">
-        <f t="shared" si="0"/>
-        <v>8500</v>
-      </c>
-    </row>
-    <row r="21" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C21" s="4" t="s">
+      <c r="D21" s="4">
+        <v>8285.8571428571431</v>
+      </c>
+    </row>
+    <row r="22" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C22" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D21" s="5">
-        <v>58001</v>
-      </c>
-      <c r="E21" s="6">
-        <f t="shared" si="0"/>
-        <v>8285.8571428571431</v>
-      </c>
-    </row>
-    <row r="22" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C22" s="4" t="s">
+      <c r="D22" s="4">
+        <v>8215</v>
+      </c>
+    </row>
+    <row r="23" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C23" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D22" s="5">
-        <v>57505</v>
-      </c>
-      <c r="E22" s="6">
-        <f t="shared" si="0"/>
-        <v>8215</v>
-      </c>
-    </row>
-    <row r="23" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C23" s="4" t="s">
+      <c r="D23" s="4">
+        <v>8142.8571428571431</v>
+      </c>
+    </row>
+    <row r="24" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C24" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D23" s="5">
-        <v>57000</v>
-      </c>
-      <c r="E23" s="6">
-        <f t="shared" si="0"/>
-        <v>8142.8571428571431</v>
-      </c>
-    </row>
-    <row r="24" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C24" s="7" t="s">
+      <c r="D24" s="4">
+        <v>8142.7142857142853</v>
+      </c>
+    </row>
+    <row r="25" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C25" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D24" s="5">
-        <v>56999</v>
-      </c>
-      <c r="E24" s="6">
-        <f t="shared" si="0"/>
-        <v>8142.7142857142853</v>
-      </c>
-    </row>
-    <row r="25" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C25" s="4" t="s">
+      <c r="D25" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="26" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C26" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D25" s="5">
-        <v>43000</v>
-      </c>
-      <c r="E25" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="26" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C26" s="4" t="s">
+      <c r="D26" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="27" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C27" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D26" s="5">
-        <v>40000</v>
-      </c>
-      <c r="E26" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="27" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C27" s="4" t="s">
+      <c r="D27" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="28" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C28" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D27" s="5">
-        <v>38000</v>
-      </c>
-      <c r="E27" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="28" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C28" s="4" t="s">
+      <c r="D28" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="29" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C29" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D28" s="5">
-        <v>37043</v>
-      </c>
-      <c r="E28" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="29" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C29" s="4" t="s">
+      <c r="D29" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="30" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C30" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D29" s="5">
-        <v>27000</v>
-      </c>
-      <c r="E29" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="30" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C30" s="4" t="s">
+      <c r="D30" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="31" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C31" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D30" s="5">
-        <v>26000</v>
-      </c>
-      <c r="E30" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="31" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C31" s="4" t="s">
+      <c r="D31" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="32" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C32" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D31" s="5">
-        <v>26000</v>
-      </c>
-      <c r="E31" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="32" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C32" s="4" t="s">
+      <c r="D32" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="33" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C33" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D32" s="5">
-        <v>26000</v>
-      </c>
-      <c r="E32" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="33" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C33" s="4" t="s">
+      <c r="D33" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="34" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C34" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D33" s="5">
-        <v>25000</v>
-      </c>
-      <c r="E33" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="34" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C34" s="4" t="s">
+      <c r="D34" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="35" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C35" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D34" s="5">
-        <v>24000</v>
-      </c>
-      <c r="E34" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="35" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C35" s="4" t="s">
+      <c r="D35" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="36" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C36" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D35" s="5">
-        <v>23000</v>
-      </c>
-      <c r="E35" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="36" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C36" s="4" t="s">
+      <c r="D36" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="37" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C37" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D36" s="5">
-        <v>22000</v>
-      </c>
-      <c r="E36" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="37" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C37" s="4" t="s">
+      <c r="D37" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="38" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C38" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D37" s="5">
-        <v>22000</v>
-      </c>
-      <c r="E37" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="38" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C38" s="4" t="s">
+      <c r="D38" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="39" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C39" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D38" s="5">
-        <v>21000</v>
-      </c>
-      <c r="E38" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="39" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C39" s="4" t="s">
+      <c r="D39" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="40" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C40" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D39" s="5">
-        <v>21000</v>
-      </c>
-      <c r="E39" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="40" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C40" s="4" t="s">
+      <c r="D40" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="41" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C41" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D40" s="5">
-        <v>21000</v>
-      </c>
-      <c r="E40" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="41" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C41" s="4" t="s">
+      <c r="D41" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="42" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C42" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D41" s="5">
-        <v>20000</v>
-      </c>
-      <c r="E41" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="42" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C42" s="4" t="s">
+      <c r="D42" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="43" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C43" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D42" s="5">
-        <v>20000</v>
-      </c>
-      <c r="E42" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="43" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C43" s="4" t="s">
+      <c r="D43" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="44" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C44" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D43" s="5">
-        <v>20000</v>
-      </c>
-      <c r="E43" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="44" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C44" s="4" t="s">
+      <c r="D44" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="45" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C45" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D44" s="5">
-        <v>19075</v>
-      </c>
-      <c r="E44" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="45" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C45" s="4" t="s">
+      <c r="D45" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="46" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C46" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D45" s="5">
-        <v>19000</v>
-      </c>
-      <c r="E45" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="46" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C46" s="4" t="s">
+      <c r="D46" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="47" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C47" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D46" s="5">
-        <v>19000</v>
-      </c>
-      <c r="E46" s="6">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="47" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C47" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D47" s="5">
-        <v>19000</v>
-      </c>
-      <c r="E47" s="6">
+      <c r="D47" s="4">
         <v>8000</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="C5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>